<commit_message>
fix: standardized model names
</commit_message>
<xml_diff>
--- a/experiments/lora_finetuning/best_models/report/best_models.xlsx
+++ b/experiments/lora_finetuning/best_models/report/best_models.xlsx
@@ -562,14 +562,14 @@
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -589,7 +589,7 @@
       <c r="F1" s="3" t="n"/>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>GPT-4o-mini</t>
+          <t>GPT</t>
         </is>
       </c>
       <c r="H1" s="2" t="n"/>
@@ -611,17 +611,17 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>Term Acc (%)</t>
+          <t>Term Accuracy %</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>Cons Macro Avg</t>
+          <t>Macro Consistency</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>Cons Weighted Avg</t>
+          <t>Weighted Consistency</t>
         </is>
       </c>
       <c r="G2" s="1" t="inlineStr">
@@ -636,17 +636,17 @@
       </c>
       <c r="I2" s="1" t="inlineStr">
         <is>
-          <t>Term Acc (%)</t>
+          <t>Term Accuracy %</t>
         </is>
       </c>
       <c r="J2" s="1" t="inlineStr">
         <is>
-          <t>Cons Macro Avg</t>
+          <t>Macro Consistency</t>
         </is>
       </c>
       <c r="K2" s="1" t="inlineStr">
         <is>
-          <t>Cons Weighted Avg</t>
+          <t>Weighted Consistency</t>
         </is>
       </c>
     </row>

</xml_diff>